<commit_message>
add test on banks import
</commit_message>
<xml_diff>
--- a/fmt/tests/banks_import.xlsx
+++ b/fmt/tests/banks_import.xlsx
@@ -91,10 +91,10 @@
     <t xml:space="preserve">https://www.abnamro.be/</t>
   </si>
   <si>
-    <t xml:space="preserve">BE0819210332</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0819210332</t>
+    <t xml:space="preserve">BE0878278532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0869211432</t>
   </si>
   <si>
     <t xml:space="preserve">ABNABE2A</t>
@@ -118,10 +118,10 @@
     <t xml:space="preserve">https://www.medirect.be/</t>
   </si>
   <si>
-    <t xml:space="preserve">BE0553851093</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0553851093</t>
+    <t xml:space="preserve">BE0569852213</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0443859893</t>
   </si>
   <si>
     <t xml:space="preserve">MBWMBEBB</t>
@@ -145,10 +145,10 @@
     <t xml:space="preserve">https://www.rabobank.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">BE0426220671</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0426220671</t>
+    <t xml:space="preserve">BE0726245271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0446220001</t>
   </si>
   <si>
     <t xml:space="preserve">RABOBE22</t>
@@ -172,10 +172,10 @@
     <t xml:space="preserve">https://www.vandeput.be/</t>
   </si>
   <si>
-    <t xml:space="preserve">BE0404501381</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0404501381</t>
+    <t xml:space="preserve">BE0804550301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0454506981</t>
   </si>
   <si>
     <t xml:space="preserve">VAPEBE22</t>
@@ -199,10 +199,10 @@
     <t xml:space="preserve">https://www.merciervanlanschot.be/</t>
   </si>
   <si>
-    <t xml:space="preserve">BE0873296641</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0873296641</t>
+    <t xml:space="preserve">BE0898297741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0153596651</t>
   </si>
   <si>
     <t xml:space="preserve">FVLBBE22</t>
@@ -220,6 +220,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -279,8 +280,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -409,247 +418,251 @@
   </sheetPr>
   <dimension ref="A1:N6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="29.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="18.49"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="2" t="n">
         <v>2600</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="M2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N2" s="0" t="s">
+      <c r="N2" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="0" t="s">
+      <c r="L3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="0" t="s">
+      <c r="M3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="0" t="s">
+      <c r="N3" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="0" t="s">
+      <c r="L4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="M4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="N4" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="K5" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L5" s="0" t="s">
+      <c r="L5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M5" s="0" t="s">
+      <c r="M5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="0" t="s">
+      <c r="N5" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="K6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="L6" s="0" t="s">
+      <c r="L6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="M6" s="0" t="s">
+      <c r="M6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="N6" s="2" t="s">
         <v>61</v>
       </c>
     </row>

</xml_diff>